<commit_message>
Firmas del Director Técnico y del Jefe en Humedad, Peso unitario y Gravedad específica fino y grueso
Además, se repara el vínculo externo que dejaba el Excel de Peso unitario (con la plantilla guardada desde Excel) como archivo dañado al abrirlo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/GDA-FLC-004_masa_unitaria.xlsx
+++ b/templates/GDA-FLC-004_masa_unitaria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GeoDelta Líneas\Dropbox\14. GEODELTA\014 FORMATOS ACTUALIZADOS 2026\FORMATOS PARA DIGITAR ACTUALIZADOS 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DCM-04\AppData\Local\Temp\claude\D--Documents-Prototipos-claude-code-interfaz\dc24a8ee-ce81-4bc3-875e-fdda07eddd40\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42148F7D-B2ED-4A6B-B7EF-CA872D74D83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E6D4DCE-686D-4E7D-9D8C-622220483CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GUIA" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">GUIA!$A$1:$K$42</definedName>
     <definedName name="GFDGSD">[1]L!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1238,53 +1238,108 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1305,8 +1360,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1316,34 +1369,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1352,51 +1379,31 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1404,69 +1411,62 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1676,14 +1676,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:f>
                       <m:fPr>
                         <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1600" i="1">
+                          <a:rPr lang="es-MX" sz="1600" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -1871,12 +1868,102 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>39956</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1484044</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Firma Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EF57C54-9F6F-4210-B39E-1A3A2A1D3A50}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect l="88188"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6497906" y="9153525"/>
+          <a:ext cx="2968088" cy="1143000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>336507</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>549318</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Firma Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7CDA13F-9398-4531-9D8C-D948F402BD90}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10709232" y="9153525"/>
+          <a:ext cx="1984461" cy="1143000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="L"/>
     </sheetNames>
@@ -2098,21 +2185,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67"/>
-      <c r="B1" s="68"/>
-      <c r="C1" s="73" t="s">
+      <c r="A1" s="82"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="75" t="s">
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="76"/>
-      <c r="K1" s="77"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="92"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="2"/>
@@ -2142,21 +2229,21 @@
       <c r="AL1" s="1"/>
     </row>
     <row r="2" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="78" t="s">
+      <c r="A2" s="84"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="82" t="s">
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="83"/>
-      <c r="K2" s="84"/>
+      <c r="J2" s="96"/>
+      <c r="K2" s="97"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="2"/>
@@ -2186,19 +2273,19 @@
       <c r="AL2" s="1"/>
     </row>
     <row r="3" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="69"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="82" t="s">
+      <c r="A3" s="84"/>
+      <c r="B3" s="85"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="83"/>
-      <c r="K3" s="84"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="97"/>
       <c r="L3" s="1"/>
       <c r="M3" s="3" t="s">
         <v>5</v>
@@ -2230,19 +2317,19 @@
       <c r="AL3" s="1"/>
     </row>
     <row r="4" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="71"/>
-      <c r="B4" s="72"/>
-      <c r="C4" s="71"/>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
-      <c r="H4" s="72"/>
-      <c r="I4" s="85" t="s">
+      <c r="A4" s="86"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="94"/>
+      <c r="E4" s="94"/>
+      <c r="F4" s="94"/>
+      <c r="G4" s="94"/>
+      <c r="H4" s="87"/>
+      <c r="I4" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="81"/>
-      <c r="K4" s="72"/>
+      <c r="J4" s="94"/>
+      <c r="K4" s="87"/>
       <c r="L4" s="1"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -2272,17 +2359,17 @@
       <c r="AL4" s="1"/>
     </row>
     <row r="5" spans="1:38" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="93"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="79"/>
-      <c r="E5" s="79"/>
-      <c r="F5" s="79"/>
-      <c r="G5" s="79"/>
-      <c r="H5" s="79"/>
-      <c r="I5" s="79"/>
-      <c r="J5" s="79"/>
-      <c r="K5" s="94"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="99"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="43"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="3"/>
@@ -2312,21 +2399,21 @@
       <c r="AL5" s="1"/>
     </row>
     <row r="6" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="95"/>
-      <c r="B6" s="96" t="s">
+      <c r="A6" s="44"/>
+      <c r="B6" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="99" t="s">
+      <c r="C6" s="100"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="60"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="98"/>
-      <c r="K6" s="101"/>
+      <c r="H6" s="103"/>
+      <c r="I6" s="104"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="105"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="4" t="s">
@@ -2358,21 +2445,21 @@
       <c r="AL6" s="1"/>
     </row>
     <row r="7" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="92"/>
-      <c r="B7" s="102" t="s">
+      <c r="A7" s="42"/>
+      <c r="B7" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="103"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
-      <c r="G7" s="104" t="s">
+      <c r="C7" s="106"/>
+      <c r="D7" s="96"/>
+      <c r="E7" s="96"/>
+      <c r="F7" s="96"/>
+      <c r="G7" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="66"/>
-      <c r="I7" s="105"/>
-      <c r="J7" s="83"/>
-      <c r="K7" s="84"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="109"/>
+      <c r="J7" s="96"/>
+      <c r="K7" s="97"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="4" t="s">
@@ -2404,21 +2491,21 @@
       <c r="AL7" s="1"/>
     </row>
     <row r="8" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="92"/>
-      <c r="B8" s="102" t="s">
+      <c r="A8" s="42"/>
+      <c r="B8" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="103"/>
-      <c r="D8" s="83"/>
-      <c r="E8" s="83"/>
-      <c r="F8" s="83"/>
-      <c r="G8" s="104" t="s">
+      <c r="C8" s="106"/>
+      <c r="D8" s="96"/>
+      <c r="E8" s="96"/>
+      <c r="F8" s="96"/>
+      <c r="G8" s="107" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="66"/>
-      <c r="I8" s="105"/>
-      <c r="J8" s="83"/>
-      <c r="K8" s="84"/>
+      <c r="H8" s="108"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="96"/>
+      <c r="K8" s="97"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1">
         <f>17-2.57</f>
@@ -2453,23 +2540,23 @@
       <c r="AL8" s="1"/>
     </row>
     <row r="9" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="92"/>
-      <c r="B9" s="102" t="s">
+      <c r="A9" s="42"/>
+      <c r="B9" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="103"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
-      <c r="G9" s="104" t="s">
+      <c r="C9" s="106"/>
+      <c r="D9" s="96"/>
+      <c r="E9" s="96"/>
+      <c r="F9" s="96"/>
+      <c r="G9" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="66"/>
-      <c r="I9" s="106" t="s">
+      <c r="H9" s="108"/>
+      <c r="I9" s="47" t="s">
         <v>18</v>
       </c>
       <c r="J9" s="5"/>
-      <c r="K9" s="107"/>
+      <c r="K9" s="48"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="4" t="s">
@@ -2501,24 +2588,24 @@
       <c r="AL9" s="1"/>
     </row>
     <row r="10" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="92"/>
-      <c r="B10" s="108" t="s">
+      <c r="A10" s="42"/>
+      <c r="B10" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="103"/>
-      <c r="D10" s="83"/>
-      <c r="E10" s="83"/>
-      <c r="F10" s="83"/>
-      <c r="G10" s="109" t="s">
+      <c r="C10" s="106"/>
+      <c r="D10" s="96"/>
+      <c r="E10" s="96"/>
+      <c r="F10" s="96"/>
+      <c r="G10" s="110" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="65"/>
-      <c r="I10" s="103" t="str">
+      <c r="H10" s="111"/>
+      <c r="I10" s="106" t="str">
         <f>CONCATENATE(J9,," ",K9,"-",D12,"-",B49,F12)</f>
         <v xml:space="preserve"> --</v>
       </c>
-      <c r="J10" s="83"/>
-      <c r="K10" s="84"/>
+      <c r="J10" s="96"/>
+      <c r="K10" s="97"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="4" t="s">
@@ -2550,17 +2637,17 @@
       <c r="AL10" s="1"/>
     </row>
     <row r="11" spans="1:38" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="110"/>
-      <c r="B11" s="111"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="45"/>
-      <c r="K11" s="112"/>
+      <c r="A11" s="50"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="113"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="51"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="4"/>
@@ -2590,25 +2677,25 @@
       <c r="AL11" s="1"/>
     </row>
     <row r="12" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="95"/>
-      <c r="B12" s="96" t="s">
+      <c r="A12" s="44"/>
+      <c r="B12" s="45" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="7"/>
-      <c r="E12" s="113" t="s">
+      <c r="E12" s="52" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="114" t="s">
         <v>25</v>
       </c>
-      <c r="H12" s="60"/>
+      <c r="H12" s="103"/>
       <c r="I12" s="9"/>
       <c r="J12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="K12" s="115"/>
+      <c r="K12" s="53"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="4"/>
@@ -2638,19 +2725,19 @@
       <c r="AL12" s="1"/>
     </row>
     <row r="13" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="92"/>
-      <c r="B13" s="102" t="s">
+      <c r="A13" s="42"/>
+      <c r="B13" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="103"/>
-      <c r="D13" s="116"/>
-      <c r="E13" s="116"/>
-      <c r="F13" s="116"/>
-      <c r="G13" s="116"/>
-      <c r="H13" s="116"/>
-      <c r="I13" s="116"/>
-      <c r="J13" s="116"/>
-      <c r="K13" s="117"/>
+      <c r="C13" s="106"/>
+      <c r="D13" s="115"/>
+      <c r="E13" s="115"/>
+      <c r="F13" s="115"/>
+      <c r="G13" s="115"/>
+      <c r="H13" s="115"/>
+      <c r="I13" s="115"/>
+      <c r="J13" s="115"/>
+      <c r="K13" s="116"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="4"/>
@@ -2680,17 +2767,17 @@
       <c r="AL13" s="1"/>
     </row>
     <row r="14" spans="1:38" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="110"/>
-      <c r="B14" s="118"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="119"/>
-      <c r="F14" s="119"/>
-      <c r="G14" s="119"/>
-      <c r="H14" s="119"/>
-      <c r="I14" s="119"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="A14" s="50"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="56"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2720,17 +2807,17 @@
       <c r="AL14" s="1"/>
     </row>
     <row r="15" spans="1:38" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="122"/>
-      <c r="F15" s="122"/>
-      <c r="G15" s="122"/>
-      <c r="H15" s="122"/>
-      <c r="I15" s="122"/>
-      <c r="J15" s="122"/>
-      <c r="K15" s="123"/>
+      <c r="A15" s="57"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="58"/>
+      <c r="J15" s="58"/>
+      <c r="K15" s="59"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
@@ -2760,19 +2847,19 @@
       <c r="AL15" s="11"/>
     </row>
     <row r="16" spans="1:38" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="124" t="s">
+      <c r="A16" s="117" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="62"/>
-      <c r="J16" s="62"/>
-      <c r="K16" s="125"/>
+      <c r="B16" s="118"/>
+      <c r="C16" s="118"/>
+      <c r="D16" s="118"/>
+      <c r="E16" s="118"/>
+      <c r="F16" s="118"/>
+      <c r="G16" s="118"/>
+      <c r="H16" s="118"/>
+      <c r="I16" s="118"/>
+      <c r="J16" s="118"/>
+      <c r="K16" s="119"/>
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
@@ -2802,17 +2889,17 @@
       <c r="AL16" s="11"/>
     </row>
     <row r="17" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="122"/>
-      <c r="F17" s="122"/>
-      <c r="G17" s="122"/>
-      <c r="H17" s="122"/>
-      <c r="I17" s="122"/>
-      <c r="J17" s="122"/>
-      <c r="K17" s="123"/>
+      <c r="A17" s="57"/>
+      <c r="B17" s="58"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="58"/>
+      <c r="K17" s="59"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
@@ -2842,25 +2929,25 @@
       <c r="AL17" s="11"/>
     </row>
     <row r="18" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="63" t="s">
+      <c r="A18" s="57"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="120" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="63" t="s">
+      <c r="E18" s="120" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="63" t="s">
+      <c r="F18" s="120" t="s">
         <v>31</v>
       </c>
-      <c r="G18" s="63" t="s">
+      <c r="G18" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="122"/>
-      <c r="I18" s="122"/>
-      <c r="J18" s="122"/>
-      <c r="K18" s="123"/>
+      <c r="H18" s="58"/>
+      <c r="I18" s="58"/>
+      <c r="J18" s="58"/>
+      <c r="K18" s="59"/>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
       <c r="N18" s="11"/>
@@ -2890,17 +2977,17 @@
       <c r="AL18" s="11"/>
     </row>
     <row r="19" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="121"/>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="64"/>
-      <c r="F19" s="64"/>
-      <c r="G19" s="64"/>
-      <c r="H19" s="122"/>
-      <c r="I19" s="122"/>
-      <c r="J19" s="122"/>
-      <c r="K19" s="123"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="121"/>
+      <c r="F19" s="121"/>
+      <c r="G19" s="121"/>
+      <c r="H19" s="58"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="58"/>
+      <c r="K19" s="59"/>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11"/>
@@ -2930,19 +3017,19 @@
       <c r="AL19" s="11"/>
     </row>
     <row r="20" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="121"/>
-      <c r="B20" s="122"/>
-      <c r="C20" s="122"/>
-      <c r="D20" s="53">
+      <c r="A20" s="57"/>
+      <c r="B20" s="58"/>
+      <c r="C20" s="58"/>
+      <c r="D20" s="122">
         <v>0</v>
       </c>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="122"/>
-      <c r="I20" s="122"/>
-      <c r="J20" s="122"/>
-      <c r="K20" s="123"/>
+      <c r="E20" s="124"/>
+      <c r="F20" s="124"/>
+      <c r="G20" s="126"/>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="59"/>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -2972,17 +3059,17 @@
       <c r="AL20" s="11"/>
     </row>
     <row r="21" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="121"/>
-      <c r="B21" s="122"/>
-      <c r="C21" s="122"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="58"/>
-      <c r="H21" s="122"/>
-      <c r="I21" s="122"/>
-      <c r="J21" s="122"/>
-      <c r="K21" s="123"/>
+      <c r="A21" s="57"/>
+      <c r="B21" s="58"/>
+      <c r="C21" s="58"/>
+      <c r="D21" s="123"/>
+      <c r="E21" s="125"/>
+      <c r="F21" s="125"/>
+      <c r="G21" s="127"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="58"/>
+      <c r="J21" s="58"/>
+      <c r="K21" s="59"/>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11"/>
@@ -3012,17 +3099,17 @@
       <c r="AL21" s="11"/>
     </row>
     <row r="22" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="121"/>
-      <c r="B22" s="122"/>
-      <c r="C22" s="122"/>
-      <c r="D22" s="122"/>
-      <c r="E22" s="122"/>
-      <c r="F22" s="122"/>
-      <c r="G22" s="122"/>
-      <c r="H22" s="122"/>
-      <c r="I22" s="122"/>
-      <c r="J22" s="122"/>
-      <c r="K22" s="123"/>
+      <c r="A22" s="57"/>
+      <c r="B22" s="58"/>
+      <c r="C22" s="58"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="58"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11"/>
@@ -3052,19 +3139,19 @@
       <c r="AL22" s="11"/>
     </row>
     <row r="23" spans="1:38" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="121"/>
-      <c r="B23" s="122"/>
-      <c r="C23" s="122"/>
-      <c r="D23" s="59" t="s">
+      <c r="A23" s="57"/>
+      <c r="B23" s="58"/>
+      <c r="C23" s="58"/>
+      <c r="D23" s="128" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="122"/>
-      <c r="I23" s="122"/>
-      <c r="J23" s="122"/>
-      <c r="K23" s="123"/>
+      <c r="E23" s="103"/>
+      <c r="F23" s="103"/>
+      <c r="G23" s="129"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="58"/>
+      <c r="K23" s="59"/>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11"/>
@@ -3094,13 +3181,13 @@
       <c r="AL23" s="11"/>
     </row>
     <row r="24" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="121"/>
-      <c r="B24" s="122"/>
-      <c r="C24" s="122"/>
-      <c r="D24" s="47" t="s">
+      <c r="A24" s="57"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="58"/>
+      <c r="D24" s="130" t="s">
         <v>34</v>
       </c>
-      <c r="E24" s="48"/>
+      <c r="E24" s="131"/>
       <c r="F24" s="12" t="s">
         <v>35</v>
       </c>
@@ -3108,10 +3195,10 @@
         <f>E20/(-(G20-D20)+F20-((F20-E20)/(L24)))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H24" s="122"/>
-      <c r="I24" s="122"/>
-      <c r="J24" s="122"/>
-      <c r="K24" s="123"/>
+      <c r="H24" s="58"/>
+      <c r="I24" s="58"/>
+      <c r="J24" s="58"/>
+      <c r="K24" s="59"/>
       <c r="L24" s="11">
         <v>0.86</v>
       </c>
@@ -3143,13 +3230,13 @@
       <c r="AL24" s="11"/>
     </row>
     <row r="25" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="121"/>
-      <c r="B25" s="122"/>
-      <c r="C25" s="122"/>
-      <c r="D25" s="49" t="s">
+      <c r="A25" s="57"/>
+      <c r="B25" s="58"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="132" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="50"/>
+      <c r="E25" s="133"/>
       <c r="F25" s="14" t="s">
         <v>35</v>
       </c>
@@ -3157,10 +3244,10 @@
         <f>G24/(1+(G28/100))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H25" s="122"/>
-      <c r="I25" s="122"/>
-      <c r="J25" s="122"/>
-      <c r="K25" s="123"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="58"/>
+      <c r="J25" s="58"/>
+      <c r="K25" s="59"/>
       <c r="L25" s="11"/>
       <c r="M25" s="11"/>
       <c r="N25" s="11"/>
@@ -3190,13 +3277,13 @@
       <c r="AL25" s="11"/>
     </row>
     <row r="26" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="121"/>
-      <c r="B26" s="122"/>
-      <c r="C26" s="122"/>
-      <c r="D26" s="49" t="s">
+      <c r="A26" s="57"/>
+      <c r="B26" s="58"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="132" t="s">
         <v>34</v>
       </c>
-      <c r="E26" s="50"/>
+      <c r="E26" s="133"/>
       <c r="F26" s="14" t="s">
         <v>37</v>
       </c>
@@ -3204,10 +3291,10 @@
         <f t="shared" ref="G26:G27" si="0">G24*10</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H26" s="122"/>
-      <c r="I26" s="122"/>
-      <c r="J26" s="122"/>
-      <c r="K26" s="123"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="59"/>
       <c r="L26" s="11"/>
       <c r="M26" s="11"/>
       <c r="N26" s="11"/>
@@ -3237,13 +3324,13 @@
       <c r="AL26" s="11"/>
     </row>
     <row r="27" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="121"/>
-      <c r="B27" s="122"/>
-      <c r="C27" s="122"/>
-      <c r="D27" s="49" t="s">
+      <c r="A27" s="57"/>
+      <c r="B27" s="58"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="132" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="50"/>
+      <c r="E27" s="133"/>
       <c r="F27" s="14" t="s">
         <v>37</v>
       </c>
@@ -3251,10 +3338,10 @@
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H27" s="122"/>
-      <c r="I27" s="122"/>
-      <c r="J27" s="122"/>
-      <c r="K27" s="123"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="58"/>
+      <c r="J27" s="58"/>
+      <c r="K27" s="59"/>
       <c r="L27" s="11"/>
       <c r="M27" s="11"/>
       <c r="N27" s="11"/>
@@ -3284,21 +3371,21 @@
       <c r="AL27" s="11"/>
     </row>
     <row r="28" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="121"/>
-      <c r="B28" s="122"/>
-      <c r="C28" s="122"/>
-      <c r="D28" s="51" t="s">
+      <c r="A28" s="57"/>
+      <c r="B28" s="58"/>
+      <c r="C28" s="58"/>
+      <c r="D28" s="134" t="s">
         <v>38</v>
       </c>
-      <c r="E28" s="52"/>
+      <c r="E28" s="135"/>
       <c r="F28" s="17" t="s">
         <v>39</v>
       </c>
       <c r="G28" s="18"/>
-      <c r="H28" s="122"/>
-      <c r="I28" s="122"/>
-      <c r="J28" s="122"/>
-      <c r="K28" s="123"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="59"/>
       <c r="L28" s="11"/>
       <c r="M28" s="11"/>
       <c r="N28" s="11"/>
@@ -3328,17 +3415,17 @@
       <c r="AL28" s="11"/>
     </row>
     <row r="29" spans="1:38" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="121"/>
-      <c r="B29" s="122"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="122"/>
-      <c r="E29" s="122"/>
-      <c r="F29" s="122"/>
-      <c r="G29" s="122"/>
-      <c r="H29" s="122"/>
-      <c r="I29" s="122"/>
-      <c r="J29" s="122"/>
-      <c r="K29" s="123"/>
+      <c r="A29" s="57"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
+      <c r="K29" s="59"/>
       <c r="L29" s="11"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11"/>
@@ -3368,19 +3455,19 @@
       <c r="AL29" s="11"/>
     </row>
     <row r="30" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="121"/>
-      <c r="B30" s="126" t="s">
+      <c r="A30" s="57"/>
+      <c r="B30" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="127"/>
-      <c r="D30" s="122"/>
-      <c r="E30" s="122"/>
-      <c r="F30" s="122"/>
-      <c r="G30" s="122"/>
-      <c r="H30" s="122"/>
-      <c r="I30" s="122"/>
-      <c r="J30" s="122"/>
-      <c r="K30" s="123"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="58"/>
+      <c r="E30" s="58"/>
+      <c r="F30" s="58"/>
+      <c r="G30" s="58"/>
+      <c r="H30" s="58"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="59"/>
       <c r="L30" s="11"/>
       <c r="M30" s="11"/>
       <c r="N30" s="11"/>
@@ -3410,21 +3497,21 @@
       <c r="AL30" s="11"/>
     </row>
     <row r="31" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="121"/>
-      <c r="B31" s="126" t="s">
+      <c r="A31" s="57"/>
+      <c r="B31" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="127"/>
-      <c r="D31" s="122"/>
-      <c r="E31" s="128" t="s">
+      <c r="C31" s="61"/>
+      <c r="D31" s="58"/>
+      <c r="E31" s="136" t="s">
         <v>42</v>
       </c>
-      <c r="F31" s="79"/>
-      <c r="G31" s="122"/>
-      <c r="H31" s="122"/>
-      <c r="I31" s="122"/>
-      <c r="J31" s="122"/>
-      <c r="K31" s="123"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="58"/>
+      <c r="J31" s="58"/>
+      <c r="K31" s="59"/>
       <c r="L31" s="11"/>
       <c r="M31" s="11"/>
       <c r="N31" s="11"/>
@@ -3454,19 +3541,19 @@
       <c r="AL31" s="11"/>
     </row>
     <row r="32" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="121"/>
-      <c r="B32" s="126" t="s">
+      <c r="A32" s="57"/>
+      <c r="B32" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="127"/>
-      <c r="D32" s="122"/>
-      <c r="E32" s="122"/>
-      <c r="F32" s="122"/>
-      <c r="G32" s="122"/>
-      <c r="H32" s="122"/>
-      <c r="I32" s="122"/>
-      <c r="J32" s="122"/>
-      <c r="K32" s="123"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="58"/>
+      <c r="G32" s="58"/>
+      <c r="H32" s="58"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="58"/>
+      <c r="K32" s="59"/>
       <c r="L32" s="11"/>
       <c r="M32" s="11"/>
       <c r="N32" s="11"/>
@@ -3496,19 +3583,19 @@
       <c r="AL32" s="11"/>
     </row>
     <row r="33" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="121"/>
-      <c r="B33" s="126" t="s">
+      <c r="A33" s="57"/>
+      <c r="B33" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="122"/>
-      <c r="D33" s="122"/>
-      <c r="E33" s="122"/>
-      <c r="F33" s="122"/>
-      <c r="G33" s="122"/>
-      <c r="H33" s="122"/>
-      <c r="I33" s="122"/>
-      <c r="J33" s="122"/>
-      <c r="K33" s="123"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58"/>
+      <c r="H33" s="58"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="58"/>
+      <c r="K33" s="59"/>
       <c r="L33" s="11"/>
       <c r="M33" s="11"/>
       <c r="N33" s="11"/>
@@ -3538,21 +3625,21 @@
       <c r="AL33" s="11"/>
     </row>
     <row r="34" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="129"/>
-      <c r="B34" s="130"/>
-      <c r="C34" s="130"/>
-      <c r="D34" s="130"/>
-      <c r="E34" s="130"/>
-      <c r="F34" s="131" t="s">
+      <c r="A34" s="62"/>
+      <c r="B34" s="63"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="72" t="s">
         <v>45</v>
       </c>
-      <c r="G34" s="79"/>
-      <c r="H34" s="132"/>
-      <c r="I34" s="131" t="s">
+      <c r="G34" s="73"/>
+      <c r="H34" s="64"/>
+      <c r="I34" s="72" t="s">
         <v>46</v>
       </c>
-      <c r="J34" s="79"/>
-      <c r="K34" s="80"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="81"/>
       <c r="L34" s="20"/>
       <c r="M34" s="20"/>
       <c r="N34" s="20"/>
@@ -3582,19 +3669,19 @@
       <c r="AL34" s="23"/>
     </row>
     <row r="35" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="133" t="s">
+      <c r="A35" s="139" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="79"/>
-      <c r="E35" s="79"/>
-      <c r="F35" s="134"/>
-      <c r="G35" s="130"/>
-      <c r="H35" s="134"/>
-      <c r="I35" s="130"/>
-      <c r="J35" s="130"/>
-      <c r="K35" s="135"/>
+      <c r="B35" s="73"/>
+      <c r="C35" s="73"/>
+      <c r="D35" s="73"/>
+      <c r="E35" s="73"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="63"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="63"/>
+      <c r="J35" s="63"/>
+      <c r="K35" s="66"/>
       <c r="L35" s="20"/>
       <c r="M35" s="11"/>
       <c r="N35" s="11"/>
@@ -3624,19 +3711,19 @@
       <c r="AL35" s="24"/>
     </row>
     <row r="36" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="136" t="s">
+      <c r="A36" s="140" t="s">
         <v>48</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="79"/>
-      <c r="D36" s="79"/>
-      <c r="E36" s="79"/>
-      <c r="F36" s="132"/>
-      <c r="G36" s="137"/>
-      <c r="H36" s="132"/>
-      <c r="I36" s="137"/>
-      <c r="J36" s="130"/>
-      <c r="K36" s="135"/>
+      <c r="B36" s="73"/>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="64"/>
+      <c r="G36" s="67"/>
+      <c r="H36" s="64"/>
+      <c r="I36" s="67"/>
+      <c r="J36" s="63"/>
+      <c r="K36" s="66"/>
       <c r="L36" s="20"/>
       <c r="M36" s="11"/>
       <c r="N36" s="11"/>
@@ -3647,9 +3734,9 @@
       <c r="S36" s="11"/>
       <c r="T36" s="20"/>
       <c r="U36" s="21"/>
-      <c r="V36" s="43"/>
-      <c r="W36" s="42"/>
-      <c r="X36" s="42"/>
+      <c r="V36" s="74"/>
+      <c r="W36" s="71"/>
+      <c r="X36" s="71"/>
       <c r="Y36" s="20"/>
       <c r="Z36" s="20"/>
       <c r="AA36" s="20"/>
@@ -3666,21 +3753,21 @@
       <c r="AL36" s="24"/>
     </row>
     <row r="37" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="69"/>
-      <c r="B37" s="79"/>
-      <c r="C37" s="79"/>
-      <c r="D37" s="79"/>
-      <c r="E37" s="79"/>
-      <c r="F37" s="138"/>
-      <c r="G37" s="130"/>
-      <c r="H37" s="138"/>
-      <c r="I37" s="130"/>
-      <c r="J37" s="130"/>
-      <c r="K37" s="135"/>
+      <c r="A37" s="84"/>
+      <c r="B37" s="73"/>
+      <c r="C37" s="73"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="68"/>
+      <c r="G37" s="63"/>
+      <c r="H37" s="68"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="66"/>
       <c r="L37" s="20"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="42"/>
-      <c r="O37" s="42"/>
+      <c r="M37" s="74"/>
+      <c r="N37" s="71"/>
+      <c r="O37" s="71"/>
       <c r="P37" s="25"/>
       <c r="Q37" s="20"/>
       <c r="R37" s="20" t="s">
@@ -3689,9 +3776,9 @@
       <c r="S37" s="20"/>
       <c r="T37" s="20"/>
       <c r="U37" s="20"/>
-      <c r="V37" s="44"/>
-      <c r="W37" s="42"/>
-      <c r="X37" s="42"/>
+      <c r="V37" s="75"/>
+      <c r="W37" s="71"/>
+      <c r="X37" s="71"/>
       <c r="Y37" s="20"/>
       <c r="Z37" s="20"/>
       <c r="AA37" s="20"/>
@@ -3708,17 +3795,17 @@
       <c r="AL37" s="24"/>
     </row>
     <row r="38" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="69"/>
-      <c r="B38" s="79"/>
-      <c r="C38" s="79"/>
-      <c r="D38" s="79"/>
-      <c r="E38" s="79"/>
-      <c r="F38" s="138"/>
-      <c r="G38" s="130"/>
-      <c r="H38" s="138"/>
-      <c r="I38" s="130"/>
-      <c r="J38" s="130"/>
-      <c r="K38" s="135"/>
+      <c r="A38" s="84"/>
+      <c r="B38" s="73"/>
+      <c r="C38" s="73"/>
+      <c r="D38" s="73"/>
+      <c r="E38" s="73"/>
+      <c r="F38" s="68"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="68"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="63"/>
+      <c r="K38" s="66"/>
       <c r="L38" s="20"/>
       <c r="M38" s="20"/>
       <c r="N38" s="20"/>
@@ -3748,35 +3835,35 @@
       <c r="AL38" s="24"/>
     </row>
     <row r="39" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="69"/>
-      <c r="B39" s="79"/>
-      <c r="C39" s="79"/>
-      <c r="D39" s="79"/>
-      <c r="E39" s="79"/>
-      <c r="F39" s="87" t="s">
+      <c r="A39" s="84"/>
+      <c r="B39" s="73"/>
+      <c r="C39" s="73"/>
+      <c r="D39" s="73"/>
+      <c r="E39" s="73"/>
+      <c r="F39" s="76" t="s">
         <v>50</v>
       </c>
-      <c r="G39" s="88"/>
-      <c r="H39" s="130"/>
-      <c r="I39" s="87" t="s">
+      <c r="G39" s="77"/>
+      <c r="H39" s="63"/>
+      <c r="I39" s="76" t="s">
         <v>66</v>
       </c>
-      <c r="J39" s="88"/>
-      <c r="K39" s="139"/>
-      <c r="L39" s="89"/>
-      <c r="M39" s="42"/>
-      <c r="N39" s="42"/>
-      <c r="O39" s="42"/>
-      <c r="P39" s="42"/>
-      <c r="Q39" s="42"/>
-      <c r="R39" s="42"/>
-      <c r="S39" s="42"/>
-      <c r="T39" s="42"/>
-      <c r="U39" s="42"/>
-      <c r="V39" s="42"/>
-      <c r="W39" s="42"/>
-      <c r="X39" s="42"/>
-      <c r="Y39" s="42"/>
+      <c r="J39" s="77"/>
+      <c r="K39" s="78"/>
+      <c r="L39" s="79"/>
+      <c r="M39" s="71"/>
+      <c r="N39" s="71"/>
+      <c r="O39" s="71"/>
+      <c r="P39" s="71"/>
+      <c r="Q39" s="71"/>
+      <c r="R39" s="71"/>
+      <c r="S39" s="71"/>
+      <c r="T39" s="71"/>
+      <c r="U39" s="71"/>
+      <c r="V39" s="71"/>
+      <c r="W39" s="71"/>
+      <c r="X39" s="71"/>
+      <c r="Y39" s="71"/>
       <c r="Z39" s="20"/>
       <c r="AA39" s="20"/>
       <c r="AB39" s="20"/>
@@ -3792,35 +3879,35 @@
       <c r="AL39" s="24"/>
     </row>
     <row r="40" spans="1:38" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="69"/>
-      <c r="B40" s="79"/>
-      <c r="C40" s="79"/>
-      <c r="D40" s="79"/>
-      <c r="E40" s="79"/>
-      <c r="F40" s="140" t="s">
+      <c r="A40" s="84"/>
+      <c r="B40" s="73"/>
+      <c r="C40" s="73"/>
+      <c r="D40" s="73"/>
+      <c r="E40" s="73"/>
+      <c r="F40" s="80" t="s">
         <v>51</v>
       </c>
-      <c r="G40" s="79"/>
-      <c r="H40" s="130"/>
-      <c r="I40" s="140" t="s">
+      <c r="G40" s="73"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="J40" s="79"/>
-      <c r="K40" s="80"/>
-      <c r="L40" s="42"/>
-      <c r="M40" s="42"/>
-      <c r="N40" s="42"/>
-      <c r="O40" s="42"/>
-      <c r="P40" s="42"/>
-      <c r="Q40" s="42"/>
-      <c r="R40" s="42"/>
-      <c r="S40" s="42"/>
-      <c r="T40" s="42"/>
-      <c r="U40" s="42"/>
-      <c r="V40" s="42"/>
-      <c r="W40" s="42"/>
-      <c r="X40" s="42"/>
-      <c r="Y40" s="42"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="71"/>
+      <c r="M40" s="71"/>
+      <c r="N40" s="71"/>
+      <c r="O40" s="71"/>
+      <c r="P40" s="71"/>
+      <c r="Q40" s="71"/>
+      <c r="R40" s="71"/>
+      <c r="S40" s="71"/>
+      <c r="T40" s="71"/>
+      <c r="U40" s="71"/>
+      <c r="V40" s="71"/>
+      <c r="W40" s="71"/>
+      <c r="X40" s="71"/>
+      <c r="Y40" s="71"/>
       <c r="Z40" s="20"/>
       <c r="AA40" s="20"/>
       <c r="AB40" s="20"/>
@@ -3836,17 +3923,17 @@
       <c r="AL40" s="24"/>
     </row>
     <row r="41" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="129"/>
-      <c r="B41" s="141"/>
-      <c r="C41" s="141"/>
-      <c r="D41" s="141"/>
-      <c r="E41" s="141"/>
-      <c r="F41" s="141"/>
-      <c r="G41" s="130"/>
-      <c r="H41" s="130"/>
-      <c r="I41" s="130"/>
-      <c r="J41" s="130"/>
-      <c r="K41" s="135"/>
+      <c r="A41" s="62"/>
+      <c r="B41" s="69"/>
+      <c r="C41" s="69"/>
+      <c r="D41" s="69"/>
+      <c r="E41" s="69"/>
+      <c r="F41" s="69"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="66"/>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
       <c r="N41" s="20"/>
@@ -3876,33 +3963,33 @@
       <c r="AL41" s="24"/>
     </row>
     <row r="42" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="142" t="s">
+      <c r="A42" s="137" t="s">
         <v>53</v>
       </c>
-      <c r="B42" s="81"/>
-      <c r="C42" s="81"/>
-      <c r="D42" s="81"/>
-      <c r="E42" s="81"/>
-      <c r="F42" s="81"/>
-      <c r="G42" s="81"/>
-      <c r="H42" s="81"/>
-      <c r="I42" s="81"/>
-      <c r="J42" s="81"/>
-      <c r="K42" s="72"/>
-      <c r="L42" s="86"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="42"/>
-      <c r="R42" s="42"/>
-      <c r="S42" s="42"/>
-      <c r="T42" s="42"/>
-      <c r="U42" s="42"/>
-      <c r="V42" s="42"/>
-      <c r="W42" s="42"/>
-      <c r="X42" s="42"/>
-      <c r="Y42" s="42"/>
+      <c r="B42" s="94"/>
+      <c r="C42" s="94"/>
+      <c r="D42" s="94"/>
+      <c r="E42" s="94"/>
+      <c r="F42" s="94"/>
+      <c r="G42" s="94"/>
+      <c r="H42" s="94"/>
+      <c r="I42" s="94"/>
+      <c r="J42" s="94"/>
+      <c r="K42" s="87"/>
+      <c r="L42" s="70"/>
+      <c r="M42" s="71"/>
+      <c r="N42" s="71"/>
+      <c r="O42" s="71"/>
+      <c r="P42" s="71"/>
+      <c r="Q42" s="71"/>
+      <c r="R42" s="71"/>
+      <c r="S42" s="71"/>
+      <c r="T42" s="71"/>
+      <c r="U42" s="71"/>
+      <c r="V42" s="71"/>
+      <c r="W42" s="71"/>
+      <c r="X42" s="71"/>
+      <c r="Y42" s="71"/>
       <c r="Z42" s="20"/>
       <c r="AA42" s="20"/>
       <c r="AB42" s="20"/>
@@ -3960,10 +4047,10 @@
     <row r="44" spans="1:38" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="20"/>
       <c r="B44" s="26"/>
-      <c r="C44" s="46" t="s">
+      <c r="C44" s="138" t="s">
         <v>54</v>
       </c>
-      <c r="D44" s="42"/>
+      <c r="D44" s="71"/>
       <c r="E44" s="26"/>
       <c r="F44" s="27" t="s">
         <v>55</v>
@@ -4004,8 +4091,8 @@
     <row r="45" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
-      <c r="C45" s="42"/>
-      <c r="D45" s="42"/>
+      <c r="C45" s="71"/>
+      <c r="D45" s="71"/>
       <c r="E45" s="30"/>
       <c r="F45" s="11"/>
       <c r="G45" s="11"/>
@@ -4044,8 +4131,8 @@
     <row r="46" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
-      <c r="C46" s="42"/>
-      <c r="D46" s="42"/>
+      <c r="C46" s="71"/>
+      <c r="D46" s="71"/>
       <c r="E46" s="30"/>
       <c r="F46" s="11"/>
       <c r="G46" s="11"/>
@@ -4084,8 +4171,8 @@
     <row r="47" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="42"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="71"/>
       <c r="E47" s="30"/>
       <c r="F47" s="11"/>
       <c r="G47" s="11"/>
@@ -4124,8 +4211,8 @@
     <row r="48" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
-      <c r="C48" s="42"/>
-      <c r="D48" s="42"/>
+      <c r="C48" s="71"/>
+      <c r="D48" s="71"/>
       <c r="E48" s="11"/>
       <c r="F48" s="11"/>
       <c r="G48" s="11"/>
@@ -4164,8 +4251,8 @@
     <row r="49" spans="1:38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
       <c r="B49" s="11"/>
-      <c r="C49" s="42"/>
-      <c r="D49" s="42"/>
+      <c r="C49" s="71"/>
+      <c r="D49" s="71"/>
       <c r="E49" s="11"/>
       <c r="F49" s="11"/>
       <c r="G49" s="11"/>
@@ -42243,6 +42330,53 @@
     </row>
   </sheetData>
   <mergeCells count="56">
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="C44:D49"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A36:E40"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="C13:K13"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="C2:H4"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="I4:K4"/>
     <mergeCell ref="L42:Y42"/>
     <mergeCell ref="F34:G34"/>
     <mergeCell ref="V36:X36"/>
@@ -42252,53 +42386,6 @@
     <mergeCell ref="I39:K39"/>
     <mergeCell ref="L39:Y40"/>
     <mergeCell ref="I40:K40"/>
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="C2:H4"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="B5:J5"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="C13:K13"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="C44:D49"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A36:E40"/>
   </mergeCells>
   <conditionalFormatting sqref="C12:D12">
     <cfRule type="containsBlanks" dxfId="4" priority="2">
@@ -42359,11 +42446,11 @@
       <c r="E4" s="31"/>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="90" t="s">
+      <c r="C5" s="141" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="91"/>
-      <c r="E5" s="91"/>
+      <c r="D5" s="142"/>
+      <c r="E5" s="142"/>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C6" s="32" t="s">

</xml_diff>